<commit_message>
fix: authority stats green bar, individual shortlink URLs, user stories
Remove green fills and date formatting from template XLSX at the XML
level. Expand generic shortlinks URL into per-community clickable links.
Add "Total" header to shortlink columns. Populate user stories section.
Find template rows by content search rather than fixed offsets.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/iznik-server/scripts/cli/authority_stats.xlsx
+++ b/iznik-server/scripts/cli/authority_stats.xlsx
@@ -271,7 +271,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="[$-809]mmm\-yy"/>
+    <numFmt numFmtId="0" formatCode="[$-809]mmm\-yy"/>
     <numFmt numFmtId="165" formatCode="&quot;£&quot;#,##0;[Red]&quot;-£&quot;#,##0"/>
     <numFmt numFmtId="166" formatCode="#,##0.0"/>
     <numFmt numFmtId="167" formatCode="&quot;£&quot;#,##0"/>
@@ -559,10 +559,7 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF17780A"/>
-        <bgColor rgb="FF17780A"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -577,10 +574,7 @@
       </patternFill>
     </fill>
     <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF17780A"/>
-        <bgColor indexed="64"/>
-      </patternFill>
+      <patternFill patternType="none"/>
     </fill>
   </fills>
   <borders count="12">
@@ -768,7 +762,7 @@
     <xf numFmtId="0" fontId="25" fillId="11" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="24" fillId="12" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -783,10 +777,10 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="26" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="26" fillId="12" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="24" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="3" fontId="24" fillId="12" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -836,16 +830,16 @@
     <xf numFmtId="0" fontId="23" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="24" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="11" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="28" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">

</xml_diff>